<commit_message>
Overhaul test fixtures with realistic FISC-compliant KB documents and add test plan
- Expand KB from 12 to 17 files with new operations/ and regulations/ categories
- Expand questionnaire from 20 to 30 questions across 12 categories
- Replace thin document content with realistic financial institution documents
  (FISC references, specific technologies, organizational structures, metrics)
- Modularize fixture content into tests/fixtures/content/ package
- Update router with new category mappings and all test assertions
- Add TEST_PLAN.md with 96 planned test additions across 6 phases

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/input/questionnaire.xlsx
+++ b/tests/fixtures/input/questionnaire.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,7 +479,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>情報セキュリティポリシーを策定・文書化していますか？また、定期的に見直しを行っていますか？</t>
+          <t>情報セキュリティポリシーの策定・承認・周知の手順と、年次見直しの実施状況を説明してください。</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -504,7 +504,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>情報セキュリティの責任者（CISO等）を任命し、責任・権限を明確にしていますか？</t>
+          <t>情報セキュリティ管理責任者（CISO等）の設置状況と、組織横断的なセキュリティ推進体制を説明してください。</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -519,17 +519,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>アクセス管理</t>
+          <t>セキュリティ管理</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ユーザー認証</t>
+          <t>リスク管理</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>システムへのアクセスにはID・パスワードによる認証を実施していますか？パスワードの複雑性要件はありますか？</t>
+          <t>情報資産のリスクアセスメント手法と実施頻度、およびリスク対応計画の策定プロセスを説明してください。</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -549,12 +549,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>権限管理</t>
+          <t>ユーザー認証</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ユーザーの権限は業務上必要最小限の範囲に制限されていますか？（最小権限の原則）</t>
+          <t>本番システムへのユーザー認証方式（多要素認証の導入状況を含む）と、認証失敗時のロックアウト設定を説明してください。</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -574,12 +574,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>特権アカウント</t>
+          <t>権限管理</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>管理者権限（特権アカウント）の利用は制限・記録されていますか？</t>
+          <t>業務システムにおけるアクセス権限の付与・変更・削除の承認フローと、定期的な棚卸しの実施状況を説明してください。</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -594,17 +594,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ウイルス対策</t>
+          <t>アクセス管理</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>マルウェア対策</t>
+          <t>特権アカウント</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>サーバー・クライアント端末にウイルス対策ソフトを導入していますか？定義ファイルの更新頻度はどうなっていますか？</t>
+          <t>特権ID（root・Administrator等）の管理方法と、利用時の承認・記録・モニタリングの仕組みを説明してください。</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -624,12 +624,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>不正プログラム</t>
+          <t>マルウェア対策</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>外部記憶媒体（USBメモリ等）の利用制限はありますか？</t>
+          <t>サーバおよび端末におけるマルウェア対策ソフトの導入状況と、パターンファイルの更新頻度を説明してください。</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -644,17 +644,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ネットワーク管理</t>
+          <t>ウイルス対策</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>境界防御</t>
+          <t>不正プログラム</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>インターネットとの接続にはファイアウォールを設置していますか？また、不要なポートは閉鎖されていますか？</t>
+          <t>未知のマルウェアや不正プログラムへの対策（EDR・サンドボックス等）の導入・運用状況を説明してください。</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -674,12 +674,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>通信暗号化</t>
+          <t>境界防御</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>外部との通信にはTLS等の暗号化プロトコルを使用していますか？</t>
+          <t>外部ネットワークとの境界におけるファイアウォール・WAF等の防御策と、ルール見直しの頻度を説明してください。</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -699,12 +699,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>不正侵入検知</t>
+          <t>通信暗号化</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IDS/IPS（不正侵入検知・防止システム）を導入していますか？</t>
+          <t>顧客データを含む通信経路における暗号化方式（TLSバージョン等）と、証明書管理の運用手順を説明してください。</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -719,17 +719,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>バックアップ管理</t>
+          <t>ネットワーク管理</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>バックアップ</t>
+          <t>不正侵入検知</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>重要データのバックアップはどのような頻度・方式で実施していますか？</t>
+          <t>IDS/IPSの導入範囲とシグネチャ更新頻度、および検知時のアラート通知・対応フローを説明してください。</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -749,12 +749,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>復旧テスト</t>
+          <t>バックアップ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>バックアップデータからの復旧テストを定期的に実施していますか？</t>
+          <t>重要データのバックアップ取得方式（フル・差分・増分）と取得頻度、遠隔地保管の実施状況を説明してください。</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -769,17 +769,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>インシデント対応</t>
+          <t>バックアップ管理</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>対応手順</t>
+          <t>復旧テスト</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>セキュリティインシデントが発生した場合の対応手順（インシデントレスポンス計画）はありますか？</t>
+          <t>バックアップからのリストアテストの実施頻度と、目標復旧時間（RTO）・復旧時点（RPO）の設定状況を説明してください。</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -799,12 +799,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>報告体制</t>
+          <t>対応手順</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>インシデント発生時の上長・関係機関への報告体制はありますか？</t>
+          <t>セキュリティインシデント発生時の初動対応手順（検知・封じ込め・根絶・復旧）の整備状況を説明してください。</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -819,17 +819,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>変更管理</t>
+          <t>インシデント対応</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>変更手順</t>
+          <t>報告体制</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>システムの変更（パッチ適用・設定変更等）に際して、変更管理手順を定めていますか？</t>
+          <t>インシデント発生時の経営層・監督官庁・顧客への報告基準とエスカレーションフローを説明してください。</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -844,17 +844,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>変更管理</t>
+          <t>インシデント対応</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>脆弱性管理</t>
+          <t>フォレンジック</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>OSやミドルウェアのセキュリティパッチは定期的に適用していますか？</t>
+          <t>デジタルフォレンジック調査の実施体制（社内・外部委託）と、証拠保全手順の整備状況を説明してください。</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -869,17 +869,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>物理セキュリティ</t>
+          <t>変更管理</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>入退室管理</t>
+          <t>変更手順</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>サーバー室等の機密エリアへの入退室管理（ICカード等）を実施していますか？</t>
+          <t>本番環境に対する変更管理プロセス（申請・承認・テスト・リリース）と、緊急変更時の手順を説明してください。</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -894,17 +894,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>物理セキュリティ</t>
+          <t>変更管理</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>設備管理</t>
+          <t>脆弱性管理</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>サーバー室の空調・電源・消火設備は整備されていますか？</t>
+          <t>OSやミドルウェアの脆弱性情報の収集体制と、セキュリティパッチ適用の優先度判断・適用手順を説明してください。</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -919,17 +919,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>教育・訓練</t>
+          <t>物理セキュリティ</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>セキュリティ教育</t>
+          <t>入退室管理</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>従業員に対して情報セキュリティ教育を定期的に実施していますか？</t>
+          <t>データセンターおよびサーバルームへの入退室管理方式（生体認証・ICカード等）と入退記録の保管期間を説明してください。</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -944,17 +944,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>教育・訓練</t>
+          <t>物理セキュリティ</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>標的型攻撃訓練</t>
+          <t>設備管理</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>フィッシングメール等の標的型攻撃を想定した訓練を実施していますか？</t>
+          <t>電源設備（UPS・自家発電）、空調設備、防火設備の冗長構成と定期点検の実施状況を説明してください。</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -963,6 +963,256 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>教育・訓練</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>セキュリティ教育</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>全従業員を対象とした情報セキュリティ教育の実施内容・頻度と、受講率の管理方法を説明してください。</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>教育・訓練</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>標的型攻撃訓練</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>標的型攻撃メール訓練の実施頻度・対象範囲と、訓練結果に基づく改善施策の実施状況を説明してください。</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>外部委託管理</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>委託先評価</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>外部委託先の選定時におけるセキュリティ評価基準と、定期的な委託先監査の実施状況を説明してください。</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>外部委託管理</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>契約管理</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>外部委託契約における秘密保持条項・セキュリティ要件・損害賠償条項の規定状況を説明してください。</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>外部委託管理</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>再委託管理</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>再委託の承認プロセスと、再委託先に対するセキュリティ管理基準の適用・監督体制を説明してください。</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>システム開発</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>開発プロセス</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>システム開発ライフサイクルにおけるセキュリティ要件定義とセキュリティレビューの実施工程を説明してください。</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>システム開発</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>コード品質</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ソースコードレビューおよび静的解析ツール（SAST）の導入状況と、指摘事項の是正管理手順を説明してください。</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>システム開発</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>脆弱性テスト</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>リリース前の脆弱性診断（DAST・ペネトレーションテスト）の実施基準と、検出された脆弱性の対応方針を説明してください。</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ログ・監視</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ログ管理</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>重要システムの操作ログ・アクセスログの取得項目、保管期間、改ざん防止策を説明してください。</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ログ・監視</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>リアルタイム監視</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SIEM等によるログの統合監視体制と、異常検知時のアラート基準・対応手順を説明してください。</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>